<commit_message>
Aggiorna Excel e HTML
</commit_message>
<xml_diff>
--- a/SonoVerse.xlsx
+++ b/SonoVerse.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matti\sonoverse-vug\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matti\Documents\sonoverse-vug\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F817CAE-016E-4DB1-BCA4-03E8F65094EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D424876E-F08F-4679-A848-AD2FF0525025}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="12864" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="100">
   <si>
     <t>Term</t>
   </si>
@@ -45,21 +45,12 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>Kidney and urinary tract</t>
-  </si>
-  <si>
     <t>Spleen</t>
   </si>
   <si>
-    <t>Ureteral jets</t>
-  </si>
-  <si>
     <t>Clip 1 B-mode</t>
   </si>
   <si>
-    <t>Metastasis target-like</t>
-  </si>
-  <si>
     <t>Gallbladder and biliary tract</t>
   </si>
   <si>
@@ -69,15 +60,6 @@
     <t>Bowel</t>
   </si>
   <si>
-    <t>Miscellaneous</t>
-  </si>
-  <si>
-    <t>Lymph nodes</t>
-  </si>
-  <si>
-    <t>Coming soon</t>
-  </si>
-  <si>
     <t xml:space="preserve">Adenomyomatosis </t>
   </si>
   <si>
@@ -87,12 +69,6 @@
     <t xml:space="preserve">Clip 1 B-mode + Color </t>
   </si>
   <si>
-    <t>Biliary hamartomatosis</t>
-  </si>
-  <si>
-    <t>Clip 1 B-mode (Convex and Linear probe)</t>
-  </si>
-  <si>
     <t>Clip 1 B-mode + Color + microV</t>
   </si>
   <si>
@@ -108,9 +84,6 @@
     <t>Adrenal adenoma</t>
   </si>
   <si>
-    <t>Intrahepatic bile ducts mild dilatation</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://youtu.be/zxTC0YBY2RY </t>
   </si>
   <si>
@@ -187,6 +160,171 @@
   </si>
   <si>
     <t>https://youtu.be/RhSUFLTmTl4</t>
+  </si>
+  <si>
+    <t>Bowel – Superior Mesenteric Artery (SMA) Syndrome</t>
+  </si>
+  <si>
+    <t>https://youtu.be/Jwjqn1j32FY</t>
+  </si>
+  <si>
+    <t>Renal angiomyolipomas</t>
+  </si>
+  <si>
+    <t>https://youtu.be/b5oGdfLmcIA</t>
+  </si>
+  <si>
+    <t>Splenic artery aneurysm</t>
+  </si>
+  <si>
+    <t>Clip 1 B-mode + Color Doppler</t>
+  </si>
+  <si>
+    <t>https://youtu.be/nKZNmbVAutI</t>
+  </si>
+  <si>
+    <t>Pancreatic adenocarcinoma (head/uncinate)</t>
+  </si>
+  <si>
+    <t>https://youtu.be/aoaF345dsKc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gallstone (Large) + Adenomyoma </t>
+  </si>
+  <si>
+    <t>https://youtu.be/mnDuOgdSpLA</t>
+  </si>
+  <si>
+    <t>Complete umbilical vein recanalization</t>
+  </si>
+  <si>
+    <t>https://youtu.be/ytNgK7wuL_M</t>
+  </si>
+  <si>
+    <t>Hepattocellular carcinoma with intra-lesional air (superinfected HCC)</t>
+  </si>
+  <si>
+    <t>https://youtu.be/4V95TgIMrbE</t>
+  </si>
+  <si>
+    <t>Parathyroid</t>
+  </si>
+  <si>
+    <t>Adenoma (primary hyperparathyroidism)</t>
+  </si>
+  <si>
+    <t>https://youtu.be/S45odD2wQOQ</t>
+  </si>
+  <si>
+    <t>Appendiceal mucocele</t>
+  </si>
+  <si>
+    <t>https://youtu.be/kdZO1IPuOIw</t>
+  </si>
+  <si>
+    <t>Severe bilateral hydronephrosis</t>
+  </si>
+  <si>
+    <t>https://youtu.be/iPGqKJn8NPs</t>
+  </si>
+  <si>
+    <t>Chronic pancreatitis: Wirsung dilatation and parenchymal calcifications</t>
+  </si>
+  <si>
+    <t>https://youtu.be/VJdnjrAAO-4</t>
+  </si>
+  <si>
+    <t>Adenomyoma</t>
+  </si>
+  <si>
+    <t>https://youtu.be/ZXwd0gwHEkQ</t>
+  </si>
+  <si>
+    <t>Budd-Chiari syndrome - Intrahepatic collateral veins</t>
+  </si>
+  <si>
+    <t>Clip 1B-mode + Color</t>
+  </si>
+  <si>
+    <t>https://youtu.be/WBORcFlYQZE</t>
+  </si>
+  <si>
+    <t>Clip 2 B-mode + Color + microV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Liver </t>
+  </si>
+  <si>
+    <t>Atypical Hemangioma - Hyperechoic with Central Hypoechoic Core</t>
+  </si>
+  <si>
+    <t>Cholesterol Crystals in Intrahepatic Bile Ducts</t>
+  </si>
+  <si>
+    <t>https://youtu.be/OvAeGcBZ--s</t>
+  </si>
+  <si>
+    <t>Aerobilia (Pneumobilia)</t>
+  </si>
+  <si>
+    <t>https://youtu.be/K2Wbg7BgXy4</t>
+  </si>
+  <si>
+    <t>Kidney</t>
+  </si>
+  <si>
+    <t>Horseshoe Kidney</t>
+  </si>
+  <si>
+    <t>https://youtu.be/wBfm-OnoUD4</t>
+  </si>
+  <si>
+    <t>Renal stone</t>
+  </si>
+  <si>
+    <t>https://youtu.be/2kRZcpi70Aw</t>
+  </si>
+  <si>
+    <t>Biliary Hamartomas (von Meyenburg Complexes)</t>
+  </si>
+  <si>
+    <t>https://youtu.be/knQhiK4Y7kY</t>
+  </si>
+  <si>
+    <t>https://youtu.be/131PwPyQ9TQ</t>
+  </si>
+  <si>
+    <t>https://youtu.be/PGVchRMB22g</t>
+  </si>
+  <si>
+    <t>Liver Steatosis with Geographic Pattern</t>
+  </si>
+  <si>
+    <t>https://youtu.be/m_H0po7LaIo</t>
+  </si>
+  <si>
+    <t>Clip 2 B-mode + Color</t>
+  </si>
+  <si>
+    <t>https://youtu.be/A3XUYC74J0o</t>
+  </si>
+  <si>
+    <t>Congestive Hepatopathy</t>
+  </si>
+  <si>
+    <t>Adrenal gland</t>
+  </si>
+  <si>
+    <t>https://youtu.be/sRu_NTopG3Y</t>
+  </si>
+  <si>
+    <t>Thyroid</t>
+  </si>
+  <si>
+    <t>Isoechoic nodule with peripheral calcifications</t>
+  </si>
+  <si>
+    <t>https://youtu.be/z_oaRVxRz5s</t>
   </si>
 </sst>
 </file>
@@ -515,11 +653,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="62.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="66.77734375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="37.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="64.21875" customWidth="1"/>
     <col min="5" max="5" width="12.109375" customWidth="1"/>
@@ -544,277 +682,575 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>63</v>
+      </c>
+      <c r="C2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
         <v>11</v>
       </c>
-      <c r="B4" t="s">
-        <v>20</v>
-      </c>
       <c r="C4" t="s">
-        <v>21</v>
+        <v>7</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>69</v>
       </c>
       <c r="C5" t="s">
-        <v>9</v>
+        <v>14</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>8</v>
+        <v>79</v>
       </c>
       <c r="C6" t="s">
-        <v>9</v>
+        <v>7</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>10</v>
+        <v>77</v>
       </c>
       <c r="C7" t="s">
-        <v>18</v>
+        <v>7</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="C8" t="s">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>32</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>3</v>
+        <v>81</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>84</v>
       </c>
       <c r="C9" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>29</v>
+        <v>85</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>3</v>
+        <v>81</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C10" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>3</v>
+        <v>81</v>
       </c>
       <c r="B11" t="s">
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="C11" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>47</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>3</v>
+        <v>81</v>
       </c>
       <c r="B12" t="s">
-        <v>52</v>
+        <v>82</v>
       </c>
       <c r="C12" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>53</v>
+        <v>83</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>37</v>
+        <v>3</v>
       </c>
       <c r="B13" t="s">
-        <v>23</v>
+        <v>86</v>
       </c>
       <c r="C13" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>38</v>
+        <v>87</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>37</v>
+        <v>3</v>
       </c>
       <c r="B14" t="s">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="C14" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>41</v>
+        <v>23</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="B15" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="C15" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="B16" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="C16" t="s">
-        <v>9</v>
+        <v>74</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>31</v>
+        <v>89</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="B17" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C17" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="B18" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C18" t="s">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="B19" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="C19" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
+        <v>3</v>
+      </c>
+      <c r="B20" t="s">
+        <v>58</v>
+      </c>
+      <c r="C20" t="s">
         <v>7</v>
       </c>
-      <c r="B20" t="s">
-        <v>33</v>
-      </c>
-      <c r="C20" t="s">
-        <v>9</v>
-      </c>
       <c r="D20" s="1" t="s">
-        <v>34</v>
+        <v>59</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
+        <v>75</v>
+      </c>
+      <c r="B21" t="s">
+        <v>76</v>
+      </c>
+      <c r="C21" t="s">
         <v>7</v>
       </c>
-      <c r="B21" t="s">
-        <v>48</v>
-      </c>
-      <c r="C21" t="s">
+      <c r="D21" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B22" t="s">
+        <v>90</v>
+      </c>
+      <c r="C22" t="s">
+        <v>7</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>28</v>
+      </c>
+      <c r="B23" t="s">
+        <v>15</v>
+      </c>
+      <c r="C23" t="s">
+        <v>16</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>28</v>
+      </c>
+      <c r="B24" t="s">
+        <v>15</v>
+      </c>
+      <c r="C24" t="s">
+        <v>92</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>28</v>
+      </c>
+      <c r="B25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" t="s">
+        <v>56</v>
+      </c>
+      <c r="C26" t="s">
+        <v>16</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>28</v>
+      </c>
+      <c r="B27" t="s">
+        <v>71</v>
+      </c>
+      <c r="C27" t="s">
+        <v>72</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>28</v>
+      </c>
+      <c r="B28" t="s">
+        <v>94</v>
+      </c>
+      <c r="C28" t="s">
+        <v>50</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>95</v>
+      </c>
+      <c r="B29" t="s">
+        <v>18</v>
+      </c>
+      <c r="C29" t="s">
+        <v>7</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
         <v>9</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="B30" t="s">
+        <v>30</v>
+      </c>
+      <c r="C30" t="s">
+        <v>7</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>9</v>
+      </c>
+      <c r="B31" t="s">
+        <v>26</v>
+      </c>
+      <c r="C31" t="s">
+        <v>14</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>9</v>
+      </c>
+      <c r="B32" t="s">
+        <v>41</v>
+      </c>
+      <c r="C32" t="s">
+        <v>16</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>9</v>
+      </c>
+      <c r="B33" t="s">
+        <v>52</v>
+      </c>
+      <c r="C33" t="s">
+        <v>16</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>9</v>
+      </c>
+      <c r="B34" t="s">
+        <v>67</v>
+      </c>
+      <c r="C34" t="s">
+        <v>16</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>60</v>
+      </c>
+      <c r="B35" t="s">
+        <v>61</v>
+      </c>
+      <c r="C35" t="s">
+        <v>16</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>6</v>
+      </c>
+      <c r="B36" t="s">
+        <v>24</v>
+      </c>
+      <c r="C36" t="s">
+        <v>7</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>6</v>
+      </c>
+      <c r="B37" t="s">
+        <v>39</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>6</v>
+      </c>
+      <c r="B38" t="s">
         <v>49</v>
       </c>
+      <c r="C38" t="s">
+        <v>50</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>97</v>
+      </c>
+      <c r="B39" t="s">
+        <v>98</v>
+      </c>
+      <c r="C39" t="s">
+        <v>16</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>99</v>
+      </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C20">
-    <sortCondition ref="A2:A20"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C36">
+    <sortCondition ref="A2:A36"/>
   </sortState>
   <hyperlinks>
-    <hyperlink ref="D3" r:id="rId1" xr:uid="{9D6B17AE-04EE-4350-A999-CB1B18813B8C}"/>
-    <hyperlink ref="D16" r:id="rId2" xr:uid="{FF4F3EC9-5254-4A3C-8F0A-334CA8AED12A}"/>
-    <hyperlink ref="D8" r:id="rId3" xr:uid="{5218EEF5-4AF3-4CD7-9F2B-5C95386BB30F}"/>
-    <hyperlink ref="D20" r:id="rId4" xr:uid="{3872027C-37FB-42D1-B676-6D4FCE37E74C}"/>
-    <hyperlink ref="D18" r:id="rId5" xr:uid="{56F5E9CD-04A6-4D7E-92FF-ADBA74D5FAE1}"/>
-    <hyperlink ref="D13" r:id="rId6" xr:uid="{A477DC1A-6E55-4652-A4B7-FA1FCF78E510}"/>
-    <hyperlink ref="D17" r:id="rId7" xr:uid="{0314C88F-1527-4D05-AE52-F4C6A7C2A550}"/>
-    <hyperlink ref="D14" r:id="rId8" xr:uid="{77275B93-2F75-42CD-8E0F-587DE257A37E}"/>
-    <hyperlink ref="D10" r:id="rId9" xr:uid="{27925F88-687C-4D84-94F8-44878BCE09D7}"/>
-    <hyperlink ref="D21" r:id="rId10" xr:uid="{FDC4E4E6-6C7E-49CC-A553-2EAC57CBEBAD}"/>
-    <hyperlink ref="D19" r:id="rId11" xr:uid="{B75AD551-422C-4496-9E1B-803AC99F34CF}"/>
-    <hyperlink ref="D12" r:id="rId12" xr:uid="{97BC6B6D-370E-4F6C-8289-D5897DCC5FED}"/>
+    <hyperlink ref="D4" r:id="rId1" xr:uid="{9D6B17AE-04EE-4350-A999-CB1B18813B8C}"/>
+    <hyperlink ref="D29" r:id="rId2" xr:uid="{FF4F3EC9-5254-4A3C-8F0A-334CA8AED12A}"/>
+    <hyperlink ref="D14" r:id="rId3" xr:uid="{5218EEF5-4AF3-4CD7-9F2B-5C95386BB30F}"/>
+    <hyperlink ref="D36" r:id="rId4" xr:uid="{3872027C-37FB-42D1-B676-6D4FCE37E74C}"/>
+    <hyperlink ref="D31" r:id="rId5" xr:uid="{56F5E9CD-04A6-4D7E-92FF-ADBA74D5FAE1}"/>
+    <hyperlink ref="D23" r:id="rId6" xr:uid="{A477DC1A-6E55-4652-A4B7-FA1FCF78E510}"/>
+    <hyperlink ref="D30" r:id="rId7" xr:uid="{0314C88F-1527-4D05-AE52-F4C6A7C2A550}"/>
+    <hyperlink ref="D25" r:id="rId8" xr:uid="{77275B93-2F75-42CD-8E0F-587DE257A37E}"/>
+    <hyperlink ref="D17" r:id="rId9" xr:uid="{27925F88-687C-4D84-94F8-44878BCE09D7}"/>
+    <hyperlink ref="D37" r:id="rId10" xr:uid="{FDC4E4E6-6C7E-49CC-A553-2EAC57CBEBAD}"/>
+    <hyperlink ref="D32" r:id="rId11" xr:uid="{B75AD551-422C-4496-9E1B-803AC99F34CF}"/>
+    <hyperlink ref="D19" r:id="rId12" xr:uid="{97BC6B6D-370E-4F6C-8289-D5897DCC5FED}"/>
+    <hyperlink ref="D3" r:id="rId13" xr:uid="{F1E9DE8C-62FD-454C-920A-6F271CC9D361}"/>
+    <hyperlink ref="D38" r:id="rId14" xr:uid="{8345F847-8095-483B-9031-E9DB791D5C93}"/>
+    <hyperlink ref="D33" r:id="rId15" xr:uid="{A5251AA5-DA3E-4368-8310-89765BD3E130}"/>
+    <hyperlink ref="D8" r:id="rId16" xr:uid="{07F90BF4-3C5C-489A-A074-E58E3F04BA37}"/>
+    <hyperlink ref="D26" r:id="rId17" xr:uid="{95CBBD08-FB80-46D1-8EA8-473BDD46FE51}"/>
+    <hyperlink ref="D20" r:id="rId18" xr:uid="{65D8AF90-619D-4C03-A962-FBDF151CA117}"/>
+    <hyperlink ref="D35" r:id="rId19" xr:uid="{CF7D7B9D-2F02-4963-B19E-FE3EAF15FE90}"/>
+    <hyperlink ref="D2" r:id="rId20" xr:uid="{8C469046-E718-48BA-BD37-48C93476C4C0}"/>
+    <hyperlink ref="D11" r:id="rId21" xr:uid="{47831B29-80C3-426B-92BE-CFB6F6A324F8}"/>
+    <hyperlink ref="D10" r:id="rId22" xr:uid="{E238BDD5-D27B-4823-B16D-362A58AE3342}"/>
+    <hyperlink ref="D34" r:id="rId23" xr:uid="{275F9260-EE59-4B3A-9E2C-CCB42C917DF6}"/>
+    <hyperlink ref="D5" r:id="rId24" xr:uid="{70369537-47F1-42B8-9BB7-46751EAC2AC8}"/>
+    <hyperlink ref="D27" r:id="rId25" xr:uid="{990E9177-F91B-48EF-9844-B1EAA6A5E520}"/>
+    <hyperlink ref="D6" r:id="rId26" xr:uid="{2ECBA23D-D340-4639-9F1A-A45FEBC5D1DC}"/>
+    <hyperlink ref="D7" r:id="rId27" xr:uid="{9AC17DC7-96F7-4112-8874-725B3D88DC74}"/>
+    <hyperlink ref="D9" r:id="rId28" xr:uid="{563947BD-F0C5-43F3-8C92-DCAA6284CDFE}"/>
+    <hyperlink ref="D13" r:id="rId29" xr:uid="{BBEDE6F8-9FD9-4D0D-BE49-3EDE31405299}"/>
+    <hyperlink ref="D21" r:id="rId30" xr:uid="{E9DF16B7-2B7E-4CE9-9338-26C71A20E0FD}"/>
+    <hyperlink ref="D22" r:id="rId31" xr:uid="{4218B645-E71B-434B-B536-5875B7968F17}"/>
+    <hyperlink ref="D24" r:id="rId32" xr:uid="{09B48A3D-0EB2-4DD4-9F2E-475294732F35}"/>
+    <hyperlink ref="D28" r:id="rId33" xr:uid="{B688936B-EA38-4943-AD32-AA81106D1883}"/>
+    <hyperlink ref="D39" r:id="rId34" xr:uid="{9A386BEF-0A88-4918-83D3-EA95C3FC2884}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>